<commit_message>
Designing Invoice Approval Part
</commit_message>
<xml_diff>
--- a/tests/projectWorkSpaceERP/finance/AP/CreatePrePaymentInvoiceData.xlsx
+++ b/tests/projectWorkSpaceERP/finance/AP/CreatePrePaymentInvoiceData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>Dataset</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>Test</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>100.10.1437.2322.90100.0000.000.0000</t>
@@ -123,7 +120,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,6 +131,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -165,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -179,8 +182,11 @@
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -190,6 +196,12 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -496,26 +508,26 @@
   <dimension ref="A1:T8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="22.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="23.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="13.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="55.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="14.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="22.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="23.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="8" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="8" width="13.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="8" width="55.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="8" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="8" width="14.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -549,7 +561,7 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
@@ -558,16 +570,16 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
@@ -611,7 +623,7 @@
       <c r="J2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="5">
         <v>1000</v>
       </c>
       <c r="L2" s="1" t="s">
@@ -620,30 +632,28 @@
       <c r="M2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2" s="6">
         <v>46113</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="1"/>
+      <c r="P2" s="6">
+        <v>46113</v>
+      </c>
+      <c r="Q2" s="6">
+        <v>46113</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="P2" s="4">
-        <v>46113</v>
-      </c>
-      <c r="Q2" s="4">
-        <v>46113</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="S2" s="1"/>
       <c r="T2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="20.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="6"/>
+      <c r="C3" s="7"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -651,13 +661,13 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="K3" s="3"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
+      <c r="N3" s="4"/>
       <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -665,7 +675,7 @@
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="20.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="6"/>
+      <c r="C4" s="7"/>
       <c r="D4" s="2"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -673,21 +683,21 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
+      <c r="K4" s="3"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
+      <c r="N4" s="4"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="20.25">
-      <c r="A5" s="6"/>
+      <c r="A5" s="7"/>
       <c r="B5" s="1"/>
-      <c r="C5" s="6"/>
+      <c r="C5" s="7"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -695,13 +705,13 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
+      <c r="K5" s="3"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
+      <c r="N5" s="4"/>
       <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
@@ -709,7 +719,7 @@
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="6"/>
+      <c r="C6" s="7"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -717,13 +727,13 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="K6" s="3"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
+      <c r="N6" s="4"/>
       <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
@@ -731,7 +741,7 @@
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="6"/>
+      <c r="C7" s="7"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -739,13 +749,13 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
+      <c r="K7" s="3"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
+      <c r="N7" s="4"/>
       <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
@@ -753,7 +763,7 @@
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="20.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="6"/>
+      <c r="C8" s="7"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -761,13 +771,13 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
+      <c r="K8" s="3"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
+      <c r="N8" s="4"/>
       <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>

</xml_diff>